<commit_message>
Implement scheme application submission modal, auto-tracking for registered mobile numbers, and live sync with Author Desk
</commit_message>
<xml_diff>
--- a/Admin_Data/User_Applications.xlsx
+++ b/Admin_Data/User_Applications.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R9"/>
+  <dimension ref="A1:R10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19" customWidth="1" min="1" max="1"/>
@@ -543,37 +543,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SS-2026-MFS-5844</t>
+          <t>SS-2026-TL-6841</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Sunita Devi</t>
+          <t>Citizen 1727</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>9888615763</t>
+          <t>9151541727</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>MFS</t>
+          <t>TL</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Micro Finance Scheme (MFS)</t>
+          <t>Term Loan</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Rs 1,25,000</t>
+          <t>₹ 150,000</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Dairy Farming and Cattle Feed</t>
+          <t>Income Generating Activity</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -596,22 +596,22 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>Application registered successfully under #SS-2026-MFS-5844. Initial document verification in progress.</t>
+          <t>Application registered for mobile #9151541727. Awaiting Scrutiny Cell review.</t>
         </is>
       </c>
       <c r="P2" t="inlineStr">
@@ -621,29 +621,29 @@
       </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-09-05 13:42:47</t>
+          <t>2026-09-06 04:19:18</t>
         </is>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>2026-09-05 13:42:47</t>
+          <t>2026-09-06 04:19:18</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SS-2026-MFS-5626</t>
+          <t>SS-2026-MFS-5844</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Test User</t>
+          <t>Sunita Devi</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>8765676029</t>
+          <t>9888615763</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -653,30 +653,30 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Micro Finance Scheme</t>
+          <t>Micro Finance Scheme (MFS)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>₹ 1,50,000</t>
+          <t>Rs 1,25,000</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Retail Kirana Shop</t>
+          <t>Dairy Farming and Cattle Feed</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>2. Document Verification</t>
+          <t>1. Application Submitted</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Under Document Verification</t>
+          <t>Application Submitted - Under Scrutiny</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -686,7 +686,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -696,34 +696,34 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>Author verified initial submission. Document verification in progress at District Scrutiny Cell.</t>
+          <t>Application registered successfully under #SS-2026-MFS-5844. Initial document verification in progress.</t>
         </is>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Keep your original Aadhaar and Caste certificates ready for verification visit.</t>
+          <t>None</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-09-04 18:09:10</t>
+          <t>2026-09-05 13:42:47</t>
         </is>
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>2026-09-05 12:35:31</t>
+          <t>2026-09-05 13:42:47</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SS-2026-MFS-2153</t>
+          <t>SS-2026-MFS-5626</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -758,15 +758,15 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>1. Application Submitted</t>
+          <t>2. Document Verification</t>
         </is>
       </c>
       <c r="I4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Application Submitted - Under Scrutiny</t>
+          <t>Under Document Verification</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -781,7 +781,7 @@
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
@@ -791,29 +791,29 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>Application registered successfully under #SS-2026-MFS-2153. Initial document verification in progress.</t>
+          <t>Author verified initial submission. Document verification in progress at District Scrutiny Cell.</t>
         </is>
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>None</t>
+          <t>Keep your original Aadhaar and Caste certificates ready for verification visit.</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-09-04 18:05:53</t>
+          <t>2026-09-04 18:09:10</t>
         </is>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>2026-09-04 18:05:53</t>
+          <t>2026-09-05 12:35:31</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SS-2026-MFS-7582</t>
+          <t>SS-2026-MFS-2153</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -881,7 +881,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>Application registered successfully under #SS-2026-MFS-7582. Initial document verification in progress.</t>
+          <t>Application registered successfully under #SS-2026-MFS-2153. Initial document verification in progress.</t>
         </is>
       </c>
       <c r="P5" t="inlineStr">
@@ -891,19 +891,19 @@
       </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-09-04 18:05:45</t>
+          <t>2026-09-04 18:05:53</t>
         </is>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>2026-09-04 18:05:45</t>
+          <t>2026-09-04 18:05:53</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SS-2026-MFS-1285</t>
+          <t>SS-2026-MFS-7582</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -971,7 +971,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>Application registered successfully under #SS-2026-MFS-1285. Initial document verification in progress.</t>
+          <t>Application registered successfully under #SS-2026-MFS-7582. Initial document verification in progress.</t>
         </is>
       </c>
       <c r="P6" t="inlineStr">
@@ -981,29 +981,29 @@
       </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>2026-09-04 18:05:36</t>
+          <t>2026-09-04 18:05:45</t>
         </is>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>2026-09-04 18:05:36</t>
+          <t>2026-09-04 18:05:45</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SS-2026-MFS-8492</t>
+          <t>SS-2026-MFS-1285</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Ramesh Chandra</t>
+          <t>Test User</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>XXXXXX4219</t>
+          <t>8765676029</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1013,30 +1013,30 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Micro Finance Scheme (MFS)</t>
+          <t>Micro Finance Scheme</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Rs 1,40,000</t>
+          <t>₹ 1,50,000</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Small Retail Kirana Store Expansion</t>
+          <t>Retail Kirana Shop</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2. Document Verification</t>
+          <t>1. Application Submitted</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Under Document Verification</t>
+          <t>Application Submitted - Under Scrutiny</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -1046,22 +1046,22 @@
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-04</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Your digital KYC and Caste certificate have been verified. Field verification by the district officer is scheduled between 05 Sep and 08 Sep 2026.</t>
+          <t>Application registered successfully under #SS-2026-MFS-1285. Initial document verification in progress.</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1071,92 +1071,92 @@
       </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2026-09-04 18:04:28</t>
+          <t>2026-09-04 18:05:36</t>
         </is>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>2026-09-04 18:04:28</t>
+          <t>2026-09-04 18:05:36</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SS-2026-ELS-3104</t>
+          <t>SS-2026-MFS-8492</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Pooja Kumari</t>
+          <t>Ramesh Chandra</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>XXXXXX8832</t>
+          <t>XXXXXX4219</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>ELS</t>
+          <t>MFS</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Educational Loan Scheme (ELS)</t>
+          <t>Micro Finance Scheme (MFS)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Rs 7,50,000</t>
+          <t>Rs 1,40,000</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>B.Tech Computer Science &amp; Engineering (4-Year Degree)</t>
+          <t>Small Retail Kirana Store Expansion</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>4. Bank Sanction</t>
+          <t>2. Document Verification</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Loan Sanctioned - Ready for Disbursement</t>
+          <t>Under Document Verification</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>APPROVED</t>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>Sanction letter #ELS-2026-9812 has been issued. Subsidized interest rate at 4.0% p.a. approved for the study tenure.</t>
+          <t>Your digital KYC and Caste certificate have been verified. Field verification by the district officer is scheduled between 05 Sep and 08 Sep 2026.</t>
         </is>
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>Please visit the branch by 06 Sep 2026 with your admission letter original and bank passbook to sign the subsidy agreement.</t>
+          <t>None</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr">
@@ -1173,88 +1173,178 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>SS-2026-ELS-3104</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Pooja Kumari</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>XXXXXX8832</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>ELS</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Educational Loan Scheme (ELS)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>Rs 7,50,000</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>B.Tech Computer Science &amp; Engineering (4-Year Degree)</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>4. Bank Sanction</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
+        <v>3</v>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Loan Sanctioned - Ready for Disbursement</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>APPROVED</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Sanction letter #ELS-2026-9812 has been issued. Subsidized interest rate at 4.0% p.a. approved for the study tenure.</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Please visit the branch by 06 Sep 2026 with your admission letter original and bank passbook to sign the subsidy agreement.</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>2026-09-04 18:04:28</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>2026-09-04 18:04:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>SS-2026-TL-5521</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>Manoj Meghwal</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>XXXXXX1904</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
+      <c r="D10" t="inlineStr">
         <is>
           <t>TERM_LOAN</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr">
+      <c r="E10" t="inlineStr">
         <is>
           <t>Term Loan (TL)</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>Rs 12,00,000</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G10" t="inlineStr">
         <is>
           <t>Food Processing &amp; Packaging Unit</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="H10" t="inlineStr">
         <is>
           <t>2. Document Verification</t>
         </is>
       </c>
-      <c r="I9" t="n">
+      <c r="I10" t="n">
         <v>1</v>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>Action Required - Document Clarification</t>
         </is>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>ACTION_REQUIRED</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>2026-08-05</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>2026-09-03</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>2026-09-22</t>
         </is>
       </c>
-      <c r="O9" t="inlineStr">
+      <c r="O10" t="inlineStr">
         <is>
           <t>Scrutiny committee found that the annual income certificate submitted was issued in 2024. As per NSFDC policy, income certificate must be valid within the past 12 months.</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
+      <c r="P10" t="inlineStr">
         <is>
           <t>Please provide an updated Family Income Certificate for FY 2026-27 issued by Tehsildar. The current document uploaded has expired.</t>
         </is>
       </c>
-      <c r="Q9" t="inlineStr">
+      <c r="Q10" t="inlineStr">
         <is>
           <t>2026-09-04 18:04:28</t>
         </is>
       </c>
-      <c r="R9" t="inlineStr">
+      <c r="R10" t="inlineStr">
         <is>
           <t>2026-09-04 18:04:28</t>
         </is>

</xml_diff>